<commit_message>
Add Southgate Office Park to marketing worksheet
The listing was added manually to real-listings.json/listing.html/map.html
but never made it into Team Utah Commercial Listings.xlsx, so a future
xlsx-to-JSON sync would have dropped it. Adds the matching FOR LEASE row.
</commit_message>
<xml_diff>
--- a/Team Utah Commercial Listings.xlsx
+++ b/Team Utah Commercial Listings.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Marketing Worksheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing Worksheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S46"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2359,345 +2359,388 @@
       <c r="S37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="4" t="n"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Southgate Office Park — 11576 State Street, Draper UT 84020</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>OFFICE</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="4" t="n">
+        <v>2650</v>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>$26.00</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Modified Gross; two 1,325 SF suites, divisible</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>https://www.crexi.com/lease/properties/1195915/utah-southgate-office-park</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="n"/>
+      <c r="L38" s="4" t="n"/>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="n"/>
+      <c r="O38" s="4" t="n"/>
+      <c r="P38" s="4" t="n"/>
+      <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>PAST PROJECTS</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>ADDRESS</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>ACRES</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>SF</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>PRICE</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>RealNex Listing</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>Offering Memorandum</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>CREXI</t>
         </is>
       </c>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>LoopNet</t>
         </is>
       </c>
-      <c r="L39" s="3" t="inlineStr">
+      <c r="L40" s="3" t="inlineStr">
         <is>
           <t>WFRMLS Link</t>
         </is>
       </c>
-      <c r="M39" s="3" t="inlineStr">
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="N39" s="3" t="inlineStr">
+      <c r="N40" s="3" t="inlineStr">
         <is>
           <t>KSL Ad Link</t>
         </is>
       </c>
-      <c r="O39" s="3" t="inlineStr">
+      <c r="O40" s="3" t="inlineStr">
         <is>
           <t>Gold Connect Link</t>
         </is>
       </c>
-      <c r="P39" s="3" t="inlineStr">
+      <c r="P40" s="3" t="inlineStr">
         <is>
           <t>Facebook Post</t>
         </is>
       </c>
-      <c r="Q39" s="3" t="inlineStr">
+      <c r="Q40" s="3" t="inlineStr">
         <is>
           <t>X post</t>
         </is>
       </c>
-      <c r="R39" s="3" t="inlineStr">
+      <c r="R40" s="3" t="inlineStr">
         <is>
           <t>Instagram Post</t>
         </is>
       </c>
-      <c r="S39" s="3" t="inlineStr">
+      <c r="S40" s="3" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr"/>
-      <c r="B40" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>1755 W North Temple, SLC - Pentecostals</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>OFFICE</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr"/>
-      <c r="E40" s="5" t="inlineStr"/>
-      <c r="F40" s="5" t="inlineStr"/>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="5" t="inlineStr"/>
-      <c r="I40" s="5" t="inlineStr"/>
-      <c r="J40" s="5" t="inlineStr"/>
-      <c r="K40" s="5" t="inlineStr"/>
-      <c r="L40" s="5" t="inlineStr"/>
-      <c r="M40" s="5" t="inlineStr"/>
-      <c r="N40" s="5" t="inlineStr"/>
-      <c r="O40" s="5" t="inlineStr"/>
-      <c r="P40" s="5" t="inlineStr"/>
-      <c r="Q40" s="5" t="inlineStr"/>
-      <c r="R40" s="5" t="inlineStr"/>
-      <c r="S40" s="5" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr"/>
+      <c r="H41" s="5" t="inlineStr"/>
+      <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr"/>
+      <c r="K41" s="5" t="inlineStr"/>
+      <c r="L41" s="5" t="inlineStr"/>
+      <c r="M41" s="5" t="inlineStr"/>
+      <c r="N41" s="5" t="inlineStr"/>
+      <c r="O41" s="5" t="inlineStr"/>
+      <c r="P41" s="5" t="inlineStr"/>
+      <c r="Q41" s="5" t="inlineStr"/>
+      <c r="R41" s="5" t="inlineStr"/>
+      <c r="S41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>3600 N Fairfield, Layton - Kihomac</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr"/>
-      <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="4" t="inlineStr"/>
-      <c r="M41" s="4" t="inlineStr"/>
-      <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr"/>
-      <c r="P41" s="4" t="inlineStr"/>
-      <c r="Q41" s="4" t="inlineStr"/>
-      <c r="R41" s="4" t="inlineStr"/>
-      <c r="S41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr"/>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr"/>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr"/>
+      <c r="N42" s="4" t="inlineStr"/>
+      <c r="O42" s="4" t="inlineStr"/>
+      <c r="P42" s="4" t="inlineStr"/>
+      <c r="Q42" s="4" t="inlineStr"/>
+      <c r="R42" s="4" t="inlineStr"/>
+      <c r="S42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>205 West 700 South CMN</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr"/>
-      <c r="D42" s="5" t="inlineStr"/>
-      <c r="E42" s="5" t="inlineStr"/>
-      <c r="F42" s="5" t="inlineStr"/>
-      <c r="G42" s="5" t="inlineStr"/>
-      <c r="H42" s="5" t="inlineStr"/>
-      <c r="I42" s="5" t="inlineStr"/>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2196359/utah-childrens-miracle-network-office-building</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr"/>
-      <c r="L42" s="5" t="inlineStr"/>
-      <c r="M42" s="5" t="inlineStr"/>
-      <c r="N42" s="5" t="inlineStr"/>
-      <c r="O42" s="5" t="inlineStr"/>
-      <c r="P42" s="5" t="inlineStr"/>
-      <c r="Q42" s="5" t="inlineStr"/>
-      <c r="R42" s="5" t="inlineStr"/>
-      <c r="S42" s="5" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr"/>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr"/>
+      <c r="M43" s="5" t="inlineStr"/>
+      <c r="N43" s="5" t="inlineStr"/>
+      <c r="O43" s="5" t="inlineStr"/>
+      <c r="P43" s="5" t="inlineStr"/>
+      <c r="Q43" s="5" t="inlineStr"/>
+      <c r="R43" s="5" t="inlineStr"/>
+      <c r="S43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>1701</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="4" t="inlineStr"/>
-      <c r="M43" s="4" t="inlineStr"/>
-      <c r="N43" s="4" t="inlineStr"/>
-      <c r="O43" s="4" t="inlineStr"/>
-      <c r="P43" s="4" t="inlineStr"/>
-      <c r="Q43" s="4" t="inlineStr"/>
-      <c r="R43" s="4" t="inlineStr"/>
-      <c r="S43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
+      <c r="M44" s="4" t="inlineStr"/>
+      <c r="N44" s="4" t="inlineStr"/>
+      <c r="O44" s="4" t="inlineStr"/>
+      <c r="P44" s="4" t="inlineStr"/>
+      <c r="Q44" s="4" t="inlineStr"/>
+      <c r="R44" s="4" t="inlineStr"/>
+      <c r="S44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Bridger</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr"/>
-      <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="5" t="inlineStr"/>
-      <c r="F44" s="5" t="inlineStr"/>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="5" t="inlineStr"/>
-      <c r="I44" s="5" t="inlineStr"/>
-      <c r="J44" s="5" t="inlineStr"/>
-      <c r="K44" s="5" t="inlineStr"/>
-      <c r="L44" s="5" t="inlineStr"/>
-      <c r="M44" s="5" t="inlineStr"/>
-      <c r="N44" s="5" t="inlineStr"/>
-      <c r="O44" s="5" t="inlineStr"/>
-      <c r="P44" s="5" t="inlineStr"/>
-      <c r="Q44" s="5" t="inlineStr"/>
-      <c r="R44" s="5" t="inlineStr"/>
-      <c r="S44" s="5" t="inlineStr"/>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr"/>
+      <c r="M45" s="5" t="inlineStr"/>
+      <c r="N45" s="5" t="inlineStr"/>
+      <c r="O45" s="5" t="inlineStr"/>
+      <c r="P45" s="5" t="inlineStr"/>
+      <c r="Q45" s="5" t="inlineStr"/>
+      <c r="R45" s="5" t="inlineStr"/>
+      <c r="S45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>LISTING PROSPECTS (Draft)</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="32" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>ADDRESS</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>TYPE</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>ACRES</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>SF</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>PRICE</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>RealNex Listing</t>
         </is>
       </c>
-      <c r="I46" s="3" t="inlineStr">
+      <c r="I47" s="3" t="inlineStr">
         <is>
           <t>Offering Memorandum</t>
         </is>
       </c>
-      <c r="J46" s="3" t="inlineStr">
+      <c r="J47" s="3" t="inlineStr">
         <is>
           <t>CREXI</t>
         </is>
       </c>
-      <c r="K46" s="3" t="inlineStr">
+      <c r="K47" s="3" t="inlineStr">
         <is>
           <t>LoopNet</t>
         </is>
       </c>
-      <c r="L46" s="3" t="inlineStr">
+      <c r="L47" s="3" t="inlineStr">
         <is>
           <t>WFRMLS Link</t>
         </is>
       </c>
-      <c r="M46" s="3" t="inlineStr">
+      <c r="M47" s="3" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="N46" s="3" t="inlineStr">
+      <c r="N47" s="3" t="inlineStr">
         <is>
           <t>KSL Ad Link</t>
         </is>
       </c>
-      <c r="O46" s="3" t="inlineStr">
+      <c r="O47" s="3" t="inlineStr">
         <is>
           <t>Gold Connect Link</t>
         </is>
       </c>
-      <c r="P46" s="3" t="inlineStr">
+      <c r="P47" s="3" t="inlineStr">
         <is>
           <t>Facebook Post</t>
         </is>
       </c>
-      <c r="Q46" s="3" t="inlineStr">
+      <c r="Q47" s="3" t="inlineStr">
         <is>
           <t>X post</t>
         </is>
       </c>
-      <c r="R46" s="3" t="inlineStr">
+      <c r="R47" s="3" t="inlineStr">
         <is>
           <t>Instagram Post</t>
         </is>
       </c>
-      <c r="S46" s="3" t="inlineStr">
+      <c r="S47" s="3" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
@@ -2705,10 +2748,10 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A45:S45"/>
+    <mergeCell ref="A46:S46"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="A31:S31"/>
-    <mergeCell ref="A38:S38"/>
+    <mergeCell ref="A39:S39"/>
     <mergeCell ref="A2:S2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>